<commit_message>
Diet contract: change protein question wording
</commit_message>
<xml_diff>
--- a/files/diet-data-contract-v1.0.1.xlsx
+++ b/files/diet-data-contract-v1.0.1.xlsx
@@ -7463,7 +7463,7 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>{지난 끼니}에 고기·생선·달걀·두부를 드셨나요?</t>
+    <t>{지난 끼니}에 단백질류(고기·생선·달걀 등)를 드셨나요?</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
@@ -23257,7 +23257,7 @@
   <sheetPr>
     <tabColor rgb="FF315A7D"/>
   </sheetPr>
-  <dimension ref="A1:D26"/>
+  <dimension ref="A1:D27"/>
   <sheetFormatPr defaultRowHeight="14"/>
   <cols>
     <col min="1" max="1" width="22.58203125" customWidth="1"/>
@@ -23504,6 +23504,28 @@
       </c>
       <c r="D26" s="16" t="s">
         <v>2507</v>
+      </c>
+    </row>
+    <row r="27" spans="1:4" ht="28">
+      <c r="A27" s="16" t="inlineStr">
+        <is>
+          <t>단백질 질문 문장 (2026-10-07)</t>
+        </is>
+      </c>
+      <c r="B27" s="16" t="inlineStr">
+        <is>
+          <t>질문 DIET-Q-06 = 「{지난 끼니}에 고기·생선·달걀·두부를 드셨나요?」</t>
+        </is>
+      </c>
+      <c r="C27" s="16" t="inlineStr">
+        <is>
+          <t>질문 DIET-Q-06 = 「{지난 끼니}에 단백질류(고기·생선·달걀 등)를 드셨나요?」. 질문 버전은 1.0.0 그대로이며 선택지·점수는 바꾸지 않음</t>
+        </is>
+      </c>
+      <c r="D27" s="16" t="inlineStr">
+        <is>
+          <t>질문 DIET-Q-06 · 참조설정데이터</t>
+        </is>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
엑셀 자동 동기화: files/diet-data-contract-v1.0.1.xlsx, files/diet-reference-config-v1.0.0.xlsx
</commit_message>
<xml_diff>
--- a/files/diet-data-contract-v1.0.1.xlsx
+++ b/files/diet-data-contract-v1.0.1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\이사라\Documents\Project_maiReport\outputs\mai-report-policy\식이\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D95292DC-7039-49BB-A977-B818C01AA149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{652C313C-F5F7-45B7-BB44-74442E7FBC0C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="38620" windowHeight="21100" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -56315,10 +56315,6 @@
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
   <si>
-    <t>자동 노출 조건은 시간대, 평일·주말, 명절·연휴만 사용한다. 명절·연휴는 달력일자 시트의 날짜(calendar_code HOLIDAY)로 판정한다. 배달·편의점·회식·카페·사무실·급식·마트·야근·여행처럼 앱이 확인하지 않는 상황 조건은 사용하지 않는다.</t>
-    <phoneticPr fontId="6" type="noConversion"/>
-  </si>
-  <si>
     <t>목표 축은 그날 회전 질문으로 고른 축과 같다. 그 축에 금지·시간·상황 필터를 통과한 문구가 없을 때만 다음 축으로 내려가며, 그 순서는 직접 선택 → 사용자 확인 진료정보 → 3개월 이내 건강검진 신호 → 일반이다. 끼니 규칙 축도 일반 축에 포함한다. 같은 질환은 직접 선택 출처로 한 번만 반영. 금지 성격은 모든 출처를 합산</t>
     <phoneticPr fontId="6" type="noConversion"/>
   </si>
@@ -56334,11 +56330,16 @@
 끼니 규칙 축 문구 14개는 목표 축이 될 수 없다고 적혀 있었음</t>
   </si>
   <si>
-    <t>달력일자 시트에 설·추석 연휴 13일(2026 설 2/16~18 · 추석 9/24~26, 2027 설 2/5~8 · 추석 9/14~16)을 넣고, 명절·연휴 문구는 이 날짜에만 나온다
+    <t>달력일자 시트 2~14행 · 구현기준 R-03 · R-08 · R-10 · 검증규칙 V-39 · V-50 · 참조설정데이터 달력일자 시트</t>
+  </si>
+  <si>
+    <t>자동 노출 조건은 시간대, 평일·주말, 명절·연휴만 사용한다. 명절·연휴는 달력일자 시트의 날짜(calendar_code HOLIDAY)로 판정한다. 그 날짜에는 그날 목표 축에서 현재 단계 이하의 명절·연휴 문구가 통과하면 다른 문구보다 먼저 쓴다. 배달·편의점·회식·카페·사무실·급식·마트·야근·여행처럼 앱이 확인하지 않는 상황 조건은 사용하지 않는다.</t>
+    <phoneticPr fontId="6" type="noConversion"/>
+  </si>
+  <si>
+    <t>달력일자 시트에 설·추석 연휴 13일(2026 설 2/16~18 · 추석 9/24~26, 2027 설 2/5~8 · 추석 9/14~16)을 넣고, 명절·연휴 문구는 이 날짜에만 나오고, 그 날짜에는 다른 문구보다 먼저 쓴다
 끼니 규칙 축도 일반 축으로 본다: 그날 질문 축 · 직접 선택 연결 축에 통과 문구가 없을 때 끼니 규칙 축 문구가 후보가 된다</t>
-  </si>
-  <si>
-    <t>달력일자 시트 2~14행 · 구현기준 R-03 · R-08 · R-10 · 검증규칙 V-39 · V-50 · 참조설정데이터 달력일자 시트</t>
+    <phoneticPr fontId="6" type="noConversion"/>
   </si>
 </sst>
 </file>
@@ -61093,18 +61094,18 @@
         <v>2709</v>
       </c>
     </row>
-    <row r="22" spans="1:4" ht="52">
+    <row r="22" spans="1:4" ht="65">
       <c r="A22" s="8" t="s">
+        <v>2731</v>
+      </c>
+      <c r="B22" s="8" t="s">
         <v>2732</v>
       </c>
-      <c r="B22" s="8" t="s">
+      <c r="C22" s="8" t="s">
+        <v>2735</v>
+      </c>
+      <c r="D22" s="8" t="s">
         <v>2733</v>
-      </c>
-      <c r="C22" s="8" t="s">
-        <v>2734</v>
-      </c>
-      <c r="D22" s="8" t="s">
-        <v>2735</v>
       </c>
     </row>
   </sheetData>
@@ -73382,7 +73383,7 @@
         <v>2452</v>
       </c>
       <c r="C39" s="29" t="s">
-        <v>2730</v>
+        <v>2729</v>
       </c>
       <c r="D39" s="5" t="s">
         <v>2562</v>
@@ -73536,7 +73537,7 @@
         <v>2588</v>
       </c>
       <c r="C50" s="29" t="s">
-        <v>2731</v>
+        <v>2730</v>
       </c>
       <c r="D50" s="5" t="s">
         <v>2589</v>
@@ -93647,7 +93648,7 @@
         <v>214</v>
       </c>
     </row>
-    <row r="9" spans="1:7" ht="37.5">
+    <row r="9" spans="1:7" ht="62.5">
       <c r="A9" s="6" t="s">
         <v>390</v>
       </c>
@@ -93661,7 +93662,7 @@
         <v>2469</v>
       </c>
       <c r="E9" s="29" t="s">
-        <v>2729</v>
+        <v>2734</v>
       </c>
       <c r="F9" s="5" t="s">
         <v>2470</v>
@@ -95767,6 +95768,15 @@
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="문서" ma:contentTypeID="0x01010011BABF6A94C35643897AD108A63C3FA9" ma:contentTypeVersion="3" ma:contentTypeDescription="새 문서를 만듭니다." ma:contentTypeScope="" ma:versionID="0dd8771f9317307737e3c0a6afa68b4c">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="47def904-0df1-4aa1-ae40-c4bd318a6de7" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="8ccd85fd4a825fc66f8c3b5a4ab7306b" ns2:_="">
     <xsd:import namespace="47def904-0df1-4aa1-ae40-c4bd318a6de7"/>
@@ -95904,15 +95914,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FA5F7BAD-F7AB-4266-8370-535EF14A9159}">
   <ds:schemaRefs>
@@ -95923,6 +95924,14 @@
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91418F39-4898-4011-9115-620418630BB5}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{FE6123CC-E6A1-4739-AA75-207000A0601B}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -95938,12 +95947,4 @@
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/internal/obd"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
-</file>
-
-<file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{91418F39-4898-4011-9115-620418630BB5}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
 </file>
</xml_diff>